<commit_message>
v1.8: templates finais aprovados + botão Com Dados conectado
- BASE_SEMANAL_VAZIO.xlsx: template em branco revisado
- BASE_SEMANAL_DADOS.xlsx: template com dados de exemplo aprovado
- baixarTemplateComDados: conectado ao arquivo estático
- Modal: textos atualizados (8 abas, descrições revisadas)
- exporter.js: código morto removido, arquivo limpo

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/BASE_SEMANAL_VAZIO.xlsx
+++ b/templates/BASE_SEMANAL_VAZIO.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trinuscapital-my.sharepoint.com/personal/mateus_monteiro_trinusco_com_br/Documents/Área de Trabalho/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trinuscapital-my.sharepoint.com/personal/mateus_monteiro_trinusco_com_br/Documents/Área de Trabalho/TEMPORARIO/SEMANAL - ENTREGA/Relatorios/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="8_{CE7D988F-984A-4A19-A89C-3C6B3BB4DF89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65ED7C34-A5BC-4BE6-BF8A-E190582E0941}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="8_{CE7D988F-984A-4A19-A89C-3C6B3BB4DF89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DAF312D-7291-4536-AB2F-810925A170D4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{73139F22-B36F-45D6-A6D6-1C2A24802F10}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{73139F22-B36F-45D6-A6D6-1C2A24802F10}"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="2" r:id="rId1"/>
@@ -22,9 +22,6 @@
     <sheet name="PARECER" sheetId="7" r:id="rId7"/>
     <sheet name="CHECKLIST" sheetId="8" r:id="rId8"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId9"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -300,11 +297,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0&quot;%&quot;"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -571,11 +568,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -598,18 +591,11 @@
     <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -626,25 +612,42 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="44" fontId="0" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -655,20 +658,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -676,7 +670,99 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="39">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="double">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="medium">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color theme="2" tint="-0.24994659260841701"/>
+        </left>
+        <right style="thin">
+          <color theme="2" tint="-0.24994659260841701"/>
+        </right>
+        <top style="thin">
+          <color theme="2" tint="-0.24994659260841701"/>
+        </top>
+        <bottom style="thin">
+          <color theme="2" tint="-0.24994659260841701"/>
+        </bottom>
+        <vertical style="thin">
+          <color theme="2" tint="-0.24994659260841701"/>
+        </vertical>
+        <horizontal style="thin">
+          <color theme="2" tint="-0.24994659260841701"/>
+        </horizontal>
+      </border>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -698,9 +784,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color rgb="FFCBD5E1"/>
@@ -708,7 +791,28 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="166" formatCode="0.0%"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -718,15 +822,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="166" formatCode="0.0%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.89999084444715716"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
       <fill>
         <patternFill patternType="solid">
@@ -772,20 +867,14 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.89999084444715716"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color rgb="FFCBD5E1"/>
         </top>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -797,9 +886,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -811,19 +897,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -832,6 +909,9 @@
           <color rgb="FFCBD5E1"/>
         </top>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -855,6 +935,9 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="thin">
           <color rgb="FFCBD5E1"/>
@@ -862,17 +945,27 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color rgb="FFCBD5E1"/>
         </top>
       </border>
     </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="TAB - MATEUS MONTEIRO" pivot="0" count="7" xr9:uid="{86089B96-72D4-41F3-8F71-AA6CD161A99D}">
+      <tableStyleElement type="wholeTable" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="totalRow" dxfId="5"/>
+      <tableStyleElement type="firstColumn" dxfId="4"/>
+      <tableStyleElement type="lastColumn" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="1"/>
+    </tableStyle>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -884,453 +977,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="CAPA"/>
-      <sheetName val="LISTAS"/>
-      <sheetName val="CONFIGURAÇÕES"/>
-      <sheetName val="UNIDADES"/>
-      <sheetName val="VISTORIAS"/>
-      <sheetName val="DELIBERAÇÕES"/>
-      <sheetName val="MFO"/>
-      <sheetName val="PARECER"/>
-      <sheetName val="CHECKLIST"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3">
-        <row r="1">
-          <cell r="A1" t="str">
-            <v>MAPA DE UNIDADES</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>ex: Bloco 1 / Torre A</v>
-          </cell>
-          <cell r="D2" t="str">
-            <v>selecione da lista ▼</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>BLOCO</v>
-          </cell>
-          <cell r="D3" t="str">
-            <v>CATEGORIA</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D4" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D5" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D6" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D7" t="str">
-            <v>Liberado</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D8" t="str">
-            <v>Restrição</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D9" t="str">
-            <v>Estoque</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D10" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D11" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D12" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D13" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D14" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D15" t="str">
-            <v>Liberado</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D16" t="str">
-            <v>Restrição</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D17" t="str">
-            <v>Estoque</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D18" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D19" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D20" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="A21" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D21" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="A22" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D22" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="A23" t="str">
-            <v>BLOCO A</v>
-          </cell>
-          <cell r="D23" t="str">
-            <v>Liberado</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="A24" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D24" t="str">
-            <v>Restrição</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="A25" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D25" t="str">
-            <v>Estoque</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="A26" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D26" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="A27" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D27" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="A28" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D28" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="A29" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D29" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="A30" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D30" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="A31" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D31" t="str">
-            <v>Liberado</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="A32" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D32" t="str">
-            <v>Restrição</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="A33" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D33" t="str">
-            <v>Estoque</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="A34" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D34" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="A35" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D35" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="A36" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D36" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="A37" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D37" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="A38" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D38" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="A39" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D39" t="str">
-            <v>Liberado</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="A40" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D40" t="str">
-            <v>Restrição</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="A41" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D41" t="str">
-            <v>Estoque</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="A42" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D42" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="A43" t="str">
-            <v>BLOCO B</v>
-          </cell>
-          <cell r="D43" t="str">
-            <v>Aprovou Vistoria</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="4">
-        <row r="2">
-          <cell r="C2" t="str">
-            <v>selecione da lista ▼</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="C3" t="str">
-            <v>STATUS</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="C4" t="str">
-            <v>Aprovada</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="C5" t="str">
-            <v>Reprovada</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="C6" t="str">
-            <v>Aprovada</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="C7" t="str">
-            <v>Não Compareceu</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="C8" t="str">
-            <v>Aprovada</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="C9" t="str">
-            <v>Aprovada</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="C10" t="str">
-            <v>Reprovada</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="C11" t="str">
-            <v>Aprovada</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="C12" t="str">
-            <v>Aprovada</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="C13" t="str">
-            <v>Aprovada</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="C14" t="str">
-            <v>Não Compareceu</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="C15" t="str">
-            <v>Aprovada</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F2585ACC-0E2E-4ED8-BB3E-76EA6662280F}" name="Tabela2" displayName="Tabela2" ref="A3:D18" totalsRowShown="0" headerRowDxfId="30" tableBorderDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F2585ACC-0E2E-4ED8-BB3E-76EA6662280F}" name="Tabela2" displayName="Tabela2" ref="A3:D18" totalsRowShown="0" headerRowDxfId="38" tableBorderDxfId="37">
   <autoFilter ref="A3:D18" xr:uid="{F2585ACC-0E2E-4ED8-BB3E-76EA6662280F}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{063EF027-97C0-45DC-B57D-9B81CAF71ECF}" name="BLOCO"/>
@@ -1338,50 +986,50 @@
     <tableColumn id="3" xr3:uid="{3CFD77EC-D1A5-413B-86EC-6C36FBA5AE02}" name="UNIDADE"/>
     <tableColumn id="4" xr3:uid="{E4D2FADC-55AD-473D-9A87-8F71BC8230E4}" name="CATEGORIA"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TAB - MATEUS MONTEIRO" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{458A5678-694D-4E94-83CF-6E60BD870641}" name="Tabela3" displayName="Tabela3" ref="A3:F9" totalsRowShown="0" tableBorderDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{458A5678-694D-4E94-83CF-6E60BD870641}" name="Tabela3" displayName="Tabela3" ref="A3:F9" totalsRowShown="0" tableBorderDxfId="36">
   <autoFilter ref="A3:F9" xr:uid="{458A5678-694D-4E94-83CF-6E60BD870641}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{72950A9C-3E35-4863-9084-A6CE9F344D72}" name="UNIDADE"/>
-    <tableColumn id="2" xr3:uid="{3596B727-6D9D-4E2C-89FE-8CDCBA202233}" name="DATA VISTORIA" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{3596B727-6D9D-4E2C-89FE-8CDCBA202233}" name="DATA VISTORIA" dataDxfId="35"/>
     <tableColumn id="3" xr3:uid="{A95BF2E4-F4F1-4F33-8144-6DFC55E35120}" name="STATUS"/>
     <tableColumn id="4" xr3:uid="{5A34127B-21B4-4046-B4DB-13EF4FB3593C}" name="MOTIVO REPROVAÇÃO"/>
-    <tableColumn id="5" xr3:uid="{77E5869C-8CE6-475C-BBAB-840DD21C257F}" name="SEMANA Nº" dataDxfId="28">
+    <tableColumn id="5" xr3:uid="{77E5869C-8CE6-475C-BBAB-840DD21C257F}" name="SEMANA Nº" dataDxfId="34">
       <calculatedColumnFormula>IF(B4="","",WEEKNUM(B4,1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{9C2729B3-DE44-4416-B68F-6F9E4E5809E5}" name="MÊS" dataDxfId="27">
+    <tableColumn id="6" xr3:uid="{9C2729B3-DE44-4416-B68F-6F9E4E5809E5}" name="MÊS" dataDxfId="33">
       <calculatedColumnFormula>IF(B4="","",TEXT(B4,"mmmm"))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TAB - MATEUS MONTEIRO" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{62E336E2-417A-491D-AC33-9C6EAA137553}" name="Tabela4" displayName="Tabela4" ref="A3:H13" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22" tableBorderDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{62E336E2-417A-491D-AC33-9C6EAA137553}" name="Tabela4" displayName="Tabela4" ref="A3:H13" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31" tableBorderDxfId="30">
   <autoFilter ref="A3:H13" xr:uid="{62E336E2-417A-491D-AC33-9C6EAA137553}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C14FAA01-C4EE-4E33-89C3-F1BB016807CC}" name="DATA CADASTRO" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{70C2469B-B101-463E-B436-C851CF43CDC5}" name="TIPO" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{0330019D-C5DA-4210-A095-A126822866E6}" name="DESCRIÇÃO" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{138E30A8-9768-4822-8572-CB0C8113E16C}" name="1º PRAZO" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{865F2461-96A9-4577-A7B6-2FDD27CFC16F}" name="PRAZO ATUAL" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{4D3D3D95-FD68-4319-8D8F-B498D9A665BD}" name="DELTA DIAS" dataDxfId="15">
+    <tableColumn id="1" xr3:uid="{C14FAA01-C4EE-4E33-89C3-F1BB016807CC}" name="DATA CADASTRO" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{70C2469B-B101-463E-B436-C851CF43CDC5}" name="TIPO" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{0330019D-C5DA-4210-A095-A126822866E6}" name="DESCRIÇÃO" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{138E30A8-9768-4822-8572-CB0C8113E16C}" name="1º PRAZO" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{865F2461-96A9-4577-A7B6-2FDD27CFC16F}" name="PRAZO ATUAL" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{4D3D3D95-FD68-4319-8D8F-B498D9A665BD}" name="DELTA DIAS" dataDxfId="24">
       <calculatedColumnFormula>IF(OR(D4="",E4=""),"",E4-D4)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{9B682D23-9E87-4A01-B9F6-7B42B460E70A}" name="RESPONSÁVEL" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{B2F555DE-A40C-41EB-88F3-5DA450B1F54C}" name="STATUS" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{9B682D23-9E87-4A01-B9F6-7B42B460E70A}" name="RESPONSÁVEL" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{B2F555DE-A40C-41EB-88F3-5DA450B1F54C}" name="STATUS" dataDxfId="8"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TAB - MATEUS MONTEIRO" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F8F9884C-064E-456B-96F9-56EBF58B73D7}" name="Tabela5" displayName="Tabela5" ref="A3:O13" totalsRowShown="0" tableBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F8F9884C-064E-456B-96F9-56EBF58B73D7}" name="Tabela5" displayName="Tabela5" ref="A3:O13" totalsRowShown="0" tableBorderDxfId="22">
   <autoFilter ref="A3:O13" xr:uid="{F8F9884C-064E-456B-96F9-56EBF58B73D7}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{1E8313BE-9FA0-4879-8027-B81F8FBE93BB}" name="DESCRIÇÃO"/>
@@ -1390,45 +1038,45 @@
     <tableColumn id="4" xr3:uid="{41230BA6-12FE-4EE6-B260-1F06EB5D23A0}" name="PAGO" dataCellStyle="Moeda"/>
     <tableColumn id="5" xr3:uid="{38E281A2-7436-41B3-A8B3-3C2FAED8EB87}" name="A PAGAR" dataCellStyle="Moeda"/>
     <tableColumn id="6" xr3:uid="{9DD6D2E0-E5A6-4391-94DB-FB1D75ADFD4B}" name="SALDO DE CONTRATOS" dataCellStyle="Moeda"/>
-    <tableColumn id="7" xr3:uid="{F110B218-CAA3-4981-9BD6-13E6AC4E6AA4}" name="COMPROMETIDO" dataDxfId="13" dataCellStyle="Moeda">
+    <tableColumn id="7" xr3:uid="{F110B218-CAA3-4981-9BD6-13E6AC4E6AA4}" name="COMPROMETIDO" dataDxfId="21" dataCellStyle="Moeda">
       <calculatedColumnFormula>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{97EAF0B3-0E84-4A89-B435-3981FFB2F514}" name="SALDO ORÇ. NOMINAL" dataDxfId="12" dataCellStyle="Moeda">
+    <tableColumn id="8" xr3:uid="{97EAF0B3-0E84-4A89-B435-3981FFB2F514}" name="SALDO ORÇ. NOMINAL" dataDxfId="20" dataCellStyle="Moeda">
       <calculatedColumnFormula>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{FA0CD418-D7D6-4FC3-94B7-2A91513C0368}" name="SALDO ORÇ. CORRIGIDO" dataDxfId="11" dataCellStyle="Moeda">
+    <tableColumn id="9" xr3:uid="{FA0CD418-D7D6-4FC3-94B7-2A91513C0368}" name="SALDO ORÇ. CORRIGIDO" dataDxfId="19" dataCellStyle="Moeda">
       <calculatedColumnFormula>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="10" xr3:uid="{EAF80F01-0CB3-4FD1-BB33-FB9D6115CEFA}" name="PREV. FINANCEIRA" dataCellStyle="Moeda"/>
-    <tableColumn id="11" xr3:uid="{269DA9F1-4E7D-4D0A-BC09-092306E7988C}" name="CUSTO AO TÉRMINO" dataDxfId="10" dataCellStyle="Moeda">
+    <tableColumn id="11" xr3:uid="{269DA9F1-4E7D-4D0A-BC09-092306E7988C}" name="CUSTO AO TÉRMINO" dataDxfId="18" dataCellStyle="Moeda">
       <calculatedColumnFormula>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{7AF55B12-3A4D-4EC4-8C23-2698A50A8A3E}" name="DESVIO NOMINAL R$" dataDxfId="9" dataCellStyle="Moeda">
+    <tableColumn id="12" xr3:uid="{7AF55B12-3A4D-4EC4-8C23-2698A50A8A3E}" name="DESVIO NOMINAL R$" dataDxfId="17" dataCellStyle="Moeda">
       <calculatedColumnFormula>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{839353B2-5D5D-43F3-84B1-D84600D46723}" name="DESVIO NOMINAL %" dataDxfId="6" dataCellStyle="Porcentagem">
+    <tableColumn id="13" xr3:uid="{839353B2-5D5D-43F3-84B1-D84600D46723}" name="DESVIO NOMINAL %" dataDxfId="16" dataCellStyle="Porcentagem">
       <calculatedColumnFormula>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{AF78D89B-B39A-40AC-A2D4-92A1DC98B99C}" name="DESVIO CORRIGIDO R$" dataDxfId="8" dataCellStyle="Moeda">
+    <tableColumn id="14" xr3:uid="{AF78D89B-B39A-40AC-A2D4-92A1DC98B99C}" name="DESVIO CORRIGIDO R$" dataDxfId="15" dataCellStyle="Moeda">
       <calculatedColumnFormula>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{06EE0D79-B353-4D14-9616-43692033788F}" name="DESVIO CORRIGIDO %" dataDxfId="7" dataCellStyle="Porcentagem">
+    <tableColumn id="15" xr3:uid="{06EE0D79-B353-4D14-9616-43692033788F}" name="DESVIO CORRIGIDO %" dataDxfId="14" dataCellStyle="Porcentagem">
       <calculatedColumnFormula>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TAB - MATEUS MONTEIRO" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{508EADF8-83F1-4C40-802D-F499104FEF5F}" name="Tabela6" displayName="Tabela6" ref="A3:I11" totalsRowShown="0" headerRowDxfId="4" tableBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{508EADF8-83F1-4C40-802D-F499104FEF5F}" name="Tabela6" displayName="Tabela6" ref="A3:I11" totalsRowShown="0" headerRowDxfId="13" tableBorderDxfId="12">
   <autoFilter ref="A3:I11" xr:uid="{508EADF8-83F1-4C40-802D-F499104FEF5F}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{5BD0F301-FFEB-4658-8A55-B5F528502825}" name="ÁREA / LOCAL"/>
     <tableColumn id="2" xr3:uid="{94F853DB-2BB8-4C20-8BF9-D689FC3F42AA}" name="ITEM"/>
-    <tableColumn id="3" xr3:uid="{0EC052FC-A359-4CA0-9AA3-487C7C0BB615}" name="1º PRAZO" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{63DDF697-8E8C-471C-8002-136301FB00D9}" name="PRAZO ATUAL" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{4C107B7B-35A5-4257-9DA3-19CE79F2719F}" name="DELTA" dataDxfId="1">
+    <tableColumn id="3" xr3:uid="{0EC052FC-A359-4CA0-9AA3-487C7C0BB615}" name="1º PRAZO" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{63DDF697-8E8C-471C-8002-136301FB00D9}" name="PRAZO ATUAL" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{4C107B7B-35A5-4257-9DA3-19CE79F2719F}" name="DELTA" dataDxfId="9">
       <calculatedColumnFormula>IF(OR(C4="",D4=""),"",D4-C4)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{F94447DE-9C90-4E58-945C-8C648E43CB6E}" name="STATUS" dataDxfId="0"/>
@@ -1436,7 +1084,7 @@
     <tableColumn id="8" xr3:uid="{EE75F888-0109-4294-BF1A-5F857D8A7BB7}" name="OBSERVAÇÃO"/>
     <tableColumn id="9" xr3:uid="{4689D7B4-5839-45E0-8439-91603DA1EE80}" name="OCULTAR"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TAB - MATEUS MONTEIRO" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1764,51 +1412,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="10" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="20" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="9" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="8" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="8" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12"/>
+      <c r="A8" s="8"/>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
+      <c r="A9" s="8"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12"/>
+      <c r="A10" s="8"/>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
+      <c r="A11" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -1825,112 +1473,112 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="11"/>
+      <c r="A1" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="25"/>
     </row>
     <row r="2" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="11"/>
+      <c r="B2" s="25"/>
     </row>
     <row r="3" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="11"/>
+      <c r="B7" s="25"/>
     </row>
     <row r="8" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="3">
         <v>45796</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="4">
         <f>IF(B8="","",B8+4)</f>
         <v>45800</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="5">
         <f>IF(B8="","",WEEKNUM(B8,1))</f>
         <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="11"/>
+      <c r="B11" s="25"/>
     </row>
     <row r="12" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="8">
-        <f>COUNTIF([1]VISTORIAS!C:C,"Aprov*")</f>
-        <v>8</v>
+      <c r="B12" s="6">
+        <f>COUNTIF(Tabela2[CATEGORIA],"Aprovou Vistoria")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="8">
-        <f>COUNTA([1]UNIDADES!A:A)-3-COUNTIF([1]UNIDADES!D:D,"*stoque*")</f>
-        <v>35</v>
+      <c r="B13" s="6">
+        <f>COUNTA(Tabela2[CATEGORIA])</f>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="7" t="str">
         <f>IF(B13=0,"",ROUND(B12/B13*100,0))</f>
-        <v>23</v>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1956,38 +1604,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
     </row>
     <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="43" t="s">
+      <c r="C2" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="43" t="s">
+      <c r="D2" s="21" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="12" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2001,7 +1649,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0B6CE350-488A-4249-A48E-0B26C2938392}">
           <x14:formula1>
             <xm:f>CONFIG!$A$4:$A$11</xm:f>
@@ -2028,32 +1676,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C2" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="15" t="s">
         <v>39</v>
       </c>
     </row>
@@ -2078,67 +1726,67 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="19"/>
-      <c r="E4" s="18" t="str">
+      <c r="B4" s="14"/>
+      <c r="E4" s="13" t="str">
         <f>IF(B4="","",WEEKNUM(B4,1))</f>
         <v/>
       </c>
-      <c r="F4" s="18" t="str">
+      <c r="F4" s="13" t="str">
         <f t="shared" ref="F4:F15" si="0">IF(B4="","",TEXT(B4,"mmmm"))</f>
         <v/>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="16"/>
-      <c r="E5" s="18" t="str">
-        <f t="shared" ref="E4:E15" si="1">IF(B5="","",WEEKNUM(B5,1))</f>
-        <v/>
-      </c>
-      <c r="F5" s="18" t="str">
+      <c r="B5" s="11"/>
+      <c r="E5" s="13" t="str">
+        <f t="shared" ref="E5:E15" si="1">IF(B5="","",WEEKNUM(B5,1))</f>
+        <v/>
+      </c>
+      <c r="F5" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="16"/>
-      <c r="E6" s="18" t="str">
+      <c r="B6" s="11"/>
+      <c r="E6" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F6" s="18" t="str">
+      <c r="F6" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="16"/>
-      <c r="E7" s="18" t="str">
+      <c r="B7" s="11"/>
+      <c r="E7" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F7" s="18" t="str">
+      <c r="F7" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="16"/>
-      <c r="E8" s="18" t="str">
+      <c r="B8" s="11"/>
+      <c r="E8" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F8" s="18" t="str">
+      <c r="F8" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="16"/>
-      <c r="E9" s="18" t="str">
+      <c r="B9" s="11"/>
+      <c r="E9" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F9" s="18" t="str">
+      <c r="F9" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -2229,206 +1877,206 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="43" t="s">
+      <c r="C2" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="43" t="s">
+      <c r="D2" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="43" t="s">
+      <c r="E2" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="F2" s="43" t="s">
+      <c r="F2" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="G2" s="43" t="s">
+      <c r="G2" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="H2" s="43" t="s">
+      <c r="H2" s="21" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="11" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="19"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="18" t="str">
+      <c r="A4" s="14"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="13" t="str">
         <f t="shared" ref="F4" si="0">IF(OR(D4="",E4=""),"",E4-D4)</f>
         <v/>
       </c>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="19"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="18" t="str">
+      <c r="A5" s="14"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="13" t="str">
         <f t="shared" ref="F5:F13" si="1">IF(OR(D5="",E5=""),"",E5-D5)</f>
         <v/>
       </c>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="19"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="18" t="str">
+      <c r="A6" s="14"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="19"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="18" t="str">
+      <c r="A7" s="14"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="19"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="18" t="str">
+      <c r="A8" s="14"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="19"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="18" t="str">
+      <c r="A9" s="14"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="18" t="str">
+      <c r="A10" s="14"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="19"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="18" t="str">
+      <c r="A11" s="14"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="19"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="18" t="str">
+      <c r="A12" s="14"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="19"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="18" t="str">
+      <c r="A13" s="14"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H13" xr:uid="{C539A5B6-A848-4042-85ED-F139907335F5}">
-      <formula1>"Em Andamento, Pendente,Não Iniciado,Cocluido"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H13" xr:uid="{4162F99D-C349-4B06-914E-31D4230FD5CF}">
+      <formula1>"Em Andamento, Pendente,Não Iniciado,Concluído"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -2461,42 +2109,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23"/>
+      <c r="O1" s="23"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="29"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -2546,401 +2194,401 @@
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="28">
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="17">
         <f>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</f>
         <v>0</v>
       </c>
-      <c r="H4" s="28">
+      <c r="H4" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="I4" s="28">
+      <c r="I4" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="J4" s="27"/>
-      <c r="K4" s="28">
+      <c r="J4" s="16"/>
+      <c r="K4" s="17">
         <f>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</f>
         <v>0</v>
       </c>
-      <c r="L4" s="28">
+      <c r="L4" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="M4" s="29">
+      <c r="M4" s="18">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</f>
         <v>0</v>
       </c>
-      <c r="N4" s="28">
+      <c r="N4" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="O4" s="30">
+      <c r="O4" s="19">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="28">
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="17">
         <f>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</f>
         <v>0</v>
       </c>
-      <c r="H5" s="28">
+      <c r="H5" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="I5" s="28">
+      <c r="I5" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="J5" s="27"/>
-      <c r="K5" s="28">
+      <c r="J5" s="16"/>
+      <c r="K5" s="17">
         <f>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</f>
         <v>0</v>
       </c>
-      <c r="L5" s="28">
+      <c r="L5" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="18">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</f>
         <v>0</v>
       </c>
-      <c r="N5" s="28">
+      <c r="N5" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="O5" s="30">
+      <c r="O5" s="19">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="28">
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="17">
         <f>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</f>
         <v>0</v>
       </c>
-      <c r="H6" s="28">
+      <c r="H6" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="I6" s="28">
+      <c r="I6" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="J6" s="27"/>
-      <c r="K6" s="28">
+      <c r="J6" s="16"/>
+      <c r="K6" s="17">
         <f>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</f>
         <v>0</v>
       </c>
-      <c r="L6" s="28">
+      <c r="L6" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="M6" s="29">
+      <c r="M6" s="18">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</f>
         <v>0</v>
       </c>
-      <c r="N6" s="28">
+      <c r="N6" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="O6" s="30">
+      <c r="O6" s="19">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="28">
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="17">
         <f>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</f>
         <v>0</v>
       </c>
-      <c r="H7" s="28">
+      <c r="H7" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="I7" s="28">
+      <c r="I7" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="J7" s="27"/>
-      <c r="K7" s="28">
+      <c r="J7" s="16"/>
+      <c r="K7" s="17">
         <f>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</f>
         <v>0</v>
       </c>
-      <c r="L7" s="28">
+      <c r="L7" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="M7" s="29">
+      <c r="M7" s="18">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</f>
         <v>0</v>
       </c>
-      <c r="N7" s="28">
+      <c r="N7" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="O7" s="30">
+      <c r="O7" s="19">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="28">
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="17">
         <f>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</f>
         <v>0</v>
       </c>
-      <c r="H8" s="28">
+      <c r="H8" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="I8" s="28">
+      <c r="I8" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="J8" s="27"/>
-      <c r="K8" s="28">
+      <c r="J8" s="16"/>
+      <c r="K8" s="17">
         <f>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</f>
         <v>0</v>
       </c>
-      <c r="L8" s="28">
+      <c r="L8" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="M8" s="29">
+      <c r="M8" s="18">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</f>
         <v>0</v>
       </c>
-      <c r="N8" s="28">
+      <c r="N8" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="O8" s="30">
+      <c r="O8" s="19">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="28">
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="17">
         <f>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</f>
         <v>0</v>
       </c>
-      <c r="H9" s="28">
+      <c r="H9" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="I9" s="28">
+      <c r="I9" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="J9" s="27"/>
-      <c r="K9" s="28">
+      <c r="J9" s="16"/>
+      <c r="K9" s="17">
         <f>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</f>
         <v>0</v>
       </c>
-      <c r="L9" s="28">
+      <c r="L9" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="M9" s="29">
+      <c r="M9" s="18">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</f>
         <v>0</v>
       </c>
-      <c r="N9" s="28">
+      <c r="N9" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="O9" s="30">
+      <c r="O9" s="19">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="28">
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="17">
         <f>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</f>
         <v>0</v>
       </c>
-      <c r="H10" s="28">
+      <c r="H10" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="I10" s="28">
+      <c r="I10" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="J10" s="27"/>
-      <c r="K10" s="28">
+      <c r="J10" s="16"/>
+      <c r="K10" s="17">
         <f>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</f>
         <v>0</v>
       </c>
-      <c r="L10" s="28">
+      <c r="L10" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="M10" s="29">
+      <c r="M10" s="18">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</f>
         <v>0</v>
       </c>
-      <c r="N10" s="28">
+      <c r="N10" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="O10" s="30">
+      <c r="O10" s="19">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="28">
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="17">
         <f>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</f>
         <v>0</v>
       </c>
-      <c r="H11" s="28">
+      <c r="H11" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="I11" s="28">
+      <c r="I11" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="J11" s="27"/>
-      <c r="K11" s="28">
+      <c r="J11" s="16"/>
+      <c r="K11" s="17">
         <f>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</f>
         <v>0</v>
       </c>
-      <c r="L11" s="28">
+      <c r="L11" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="M11" s="29">
+      <c r="M11" s="18">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</f>
         <v>0</v>
       </c>
-      <c r="N11" s="28">
+      <c r="N11" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="O11" s="30">
+      <c r="O11" s="19">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="28">
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="17">
         <f>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</f>
         <v>0</v>
       </c>
-      <c r="H12" s="28">
+      <c r="H12" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="I12" s="28">
+      <c r="I12" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="J12" s="27"/>
-      <c r="K12" s="28">
+      <c r="J12" s="16"/>
+      <c r="K12" s="17">
         <f>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</f>
         <v>0</v>
       </c>
-      <c r="L12" s="28">
+      <c r="L12" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="M12" s="29">
+      <c r="M12" s="18">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</f>
         <v>0</v>
       </c>
-      <c r="N12" s="28">
+      <c r="N12" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="O12" s="30">
+      <c r="O12" s="19">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="27"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="28">
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="17">
         <f>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</f>
         <v>0</v>
       </c>
-      <c r="H13" s="28">
+      <c r="H13" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="I13" s="28">
+      <c r="I13" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</f>
         <v>0</v>
       </c>
-      <c r="J13" s="27"/>
-      <c r="K13" s="28">
+      <c r="J13" s="16"/>
+      <c r="K13" s="17">
         <f>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</f>
         <v>0</v>
       </c>
-      <c r="L13" s="28">
+      <c r="L13" s="17">
         <f>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="M13" s="29">
+      <c r="M13" s="18">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</f>
         <v>0</v>
       </c>
-      <c r="N13" s="28">
+      <c r="N13" s="17">
         <f>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</f>
         <v>0</v>
       </c>
-      <c r="O13" s="30">
+      <c r="O13" s="19">
         <f>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</f>
         <v>0</v>
       </c>
@@ -2966,128 +2614,128 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="23"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="32"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="31"/>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="33"/>
+      <c r="A3" s="33"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="35"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="34"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="35"/>
+      <c r="A4" s="36"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="37"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="34"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="35"/>
+      <c r="A5" s="36"/>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="37"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="34"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="35"/>
+      <c r="A6" s="36"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="37"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="34"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="35"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="37"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="34"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="35"/>
+      <c r="A8" s="36"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="37"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="34"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="35"/>
+      <c r="A9" s="36"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="37"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="34"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="35"/>
+      <c r="A10" s="36"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="37"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="34"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="35"/>
+      <c r="A11" s="36"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="37"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="34"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="35"/>
+      <c r="A12" s="36"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="37"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="34"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="35"/>
+      <c r="A13" s="36"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="37"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="34"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="35"/>
+      <c r="A14" s="36"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="37"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="34"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="35"/>
+      <c r="A15" s="36"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="37"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="34"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="35"/>
+      <c r="A16" s="36"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="37"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="34"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="35"/>
+      <c r="A17" s="36"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="37"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="34"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="35"/>
+      <c r="A18" s="36"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="37"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="34"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="35"/>
+      <c r="A19" s="36"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="37"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="36"/>
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="38"/>
+      <c r="A20" s="38"/>
+      <c r="B20" s="39"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3116,131 +2764,131 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="41" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="11" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="18" t="str">
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="13" t="str">
         <f t="shared" ref="E4:E11" si="0">IF(OR(C4="",D4=""),"",D4-C4)</f>
         <v/>
       </c>
-      <c r="F4" s="16"/>
+      <c r="F4" s="11"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="18" t="str">
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="F5" s="16"/>
+      <c r="F5" s="11"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="18" t="str">
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="F6" s="16"/>
+      <c r="F6" s="11"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="18" t="str">
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="F7" s="16"/>
+      <c r="F7" s="11"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="18" t="str">
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="F8" s="16"/>
+      <c r="F8" s="11"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="18" t="str">
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="F9" s="16"/>
+      <c r="F9" s="11"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="18" t="str">
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="F10" s="16"/>
+      <c r="F10" s="11"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="18" t="str">
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="F11" s="16"/>
+      <c r="F11" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3248,11 +2896,11 @@
     <mergeCell ref="A1:I1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F11" xr:uid="{51BD162F-C4B1-4AE0-AB7E-2F1189F611E7}">
-      <formula1>"Em Andamento, Pendente,Não Iniciado,Cocluido"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4:I11" xr:uid="{F7C6F5B1-74D2-4521-B502-E5D422E00BEE}">
       <formula1>"SIM"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F11" xr:uid="{6151D856-44E1-4051-BBF7-1E94A62D05CA}">
+      <formula1>"Em Andamento, Pendente,Não Iniciado,Concluído"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
templates: adiciona categoria REPROVADO no mapa de unidades
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/BASE_SEMANAL_VAZIO.xlsx
+++ b/templates/BASE_SEMANAL_VAZIO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trinuscapital-my.sharepoint.com/personal/mateus_monteiro_trinusco_com_br/Documents/Área de Trabalho/TEMPORARIO/SEMANAL - ENTREGA/Relatorios/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="85" documentId="11_C7687B5054A33544D9B01B6F03B42F07F57BE01D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E9BBD8D-2812-48DC-A346-7BC2B2B64C8D}"/>
+  <xr:revisionPtr revIDLastSave="86" documentId="11_C7687B5054A33544D9B01B6F03B42F07F57BE01D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCC5D997-E47E-4875-AE00-723AD7C396CB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="80">
   <si>
     <t>CHECKLIST DE ÁREA COMUM</t>
   </si>
@@ -277,6 +277,9 @@
   </si>
   <si>
     <t>Ex: 25/01/2026</t>
+  </si>
+  <si>
+    <t>Reprovado</t>
   </si>
 </sst>
 </file>
@@ -604,14 +607,17 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -632,9 +638,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -653,36 +656,6 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.89999084444715716"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color rgb="FFCBD5E1"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="165" formatCode="0.0%"/>
       <fill>
         <patternFill patternType="solid">
@@ -855,6 +828,36 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FFCBD5E1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom"/>
     </dxf>
     <dxf>
       <fill>
@@ -969,7 +972,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela2" displayName="Tabela2" ref="A3:D6" totalsRowShown="0" headerRowDxfId="35" tableBorderDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela2" displayName="Tabela2" ref="A3:D6" totalsRowShown="0" headerRowDxfId="29" tableBorderDxfId="28">
   <autoFilter ref="A3:D6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="BLOCO"/>
@@ -982,20 +985,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabela3" displayName="Tabela3" ref="A3:F6" totalsRowShown="0" tableBorderDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabela3" displayName="Tabela3" ref="A3:F6" totalsRowShown="0" tableBorderDxfId="27">
   <autoFilter ref="A3:F6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:F6">
     <sortCondition ref="B3:B6"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="UNIDADE"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="DATA VISTORIA" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="DATA VISTORIA" dataDxfId="26"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="STATUS"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="MOTIVO REPROVAÇÃO"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="SEMANA Nº" dataDxfId="31">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="SEMANA Nº" dataDxfId="25">
       <calculatedColumnFormula>IF(B4="","",WEEKNUM(B4,1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="MÊS" dataDxfId="30">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="MÊS" dataDxfId="24">
       <calculatedColumnFormula>IF(B4="","",TEXT(B4,"mmmm"))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1004,58 +1007,58 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabela4" displayName="Tabela4" ref="A3:I6" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28" tableBorderDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabela4" displayName="Tabela4" ref="A3:I6" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22" tableBorderDxfId="21">
   <autoFilter ref="A3:I6" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="DATA CADASTRO" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="TIPO" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="DESCRIÇÃO" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="1º PRAZO" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="PRAZO ATUAL" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="DELTA DIAS" dataDxfId="21">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="DATA CADASTRO" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="TIPO" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="DESCRIÇÃO" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="1º PRAZO" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="PRAZO ATUAL" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="DELTA DIAS" dataDxfId="15">
       <calculatedColumnFormula>IF(OR(D4="",E4=""),"",E4-D4)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="RESPONSÁVEL" dataDxfId="20"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="STATUS" dataDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{6816C52C-219B-44C5-9460-FB46A53D1694}" name="OCULTAR" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="RESPONSÁVEL" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="STATUS" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{6816C52C-219B-44C5-9460-FB46A53D1694}" name="OCULTAR" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TAB - MATEUS MONTEIRO" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Tabela5" displayName="Tabela5" ref="A3:O7" totalsRowShown="0" headerRowDxfId="17" tableBorderDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Tabela5" displayName="Tabela5" ref="A3:O7" totalsRowShown="0" headerRowDxfId="11" tableBorderDxfId="10">
   <autoFilter ref="A3:O7" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="DESCRIÇÃO"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="VALOR ORÇADO" dataCellStyle="Moeda"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="VALOR ATUALIZADO" dataDxfId="15" dataCellStyle="Moeda"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="VALOR ATUALIZADO" dataDxfId="9" dataCellStyle="Moeda"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="PAGO" dataCellStyle="Moeda"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="A PAGAR" dataCellStyle="Moeda"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="SALDO DE CONTRATOS" dataCellStyle="Moeda"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="COMPROMETIDO" dataDxfId="14" dataCellStyle="Moeda">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="COMPROMETIDO" dataDxfId="8" dataCellStyle="Moeda">
       <calculatedColumnFormula>SUM(Tabela5[[#This Row],[PAGO]:[SALDO DE CONTRATOS]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="SALDO ORÇ. NOMINAL" dataDxfId="13" dataCellStyle="Moeda">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="SALDO ORÇ. NOMINAL" dataDxfId="7" dataCellStyle="Moeda">
       <calculatedColumnFormula>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="SALDO ORÇ. CORRIGIDO" dataDxfId="12" dataCellStyle="Moeda">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="SALDO ORÇ. CORRIGIDO" dataDxfId="6" dataCellStyle="Moeda">
       <calculatedColumnFormula>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[COMPROMETIDO]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="PREV. FINANCEIRA" dataCellStyle="Moeda"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="CUSTO AO TÉRMINO" dataDxfId="11" dataCellStyle="Moeda">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="CUSTO AO TÉRMINO" dataDxfId="5" dataCellStyle="Moeda">
       <calculatedColumnFormula>Tabela5[[#This Row],[PREV. FINANCEIRA]]+Tabela5[[#This Row],[PAGO]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="DESVIO NOMINAL R$" dataDxfId="10" dataCellStyle="Moeda">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="DESVIO NOMINAL R$" dataDxfId="4" dataCellStyle="Moeda">
       <calculatedColumnFormula>Tabela5[[#This Row],[VALOR ORÇADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0300-00000D000000}" name="DESVIO NOMINAL %" dataDxfId="9" dataCellStyle="Porcentagem">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0300-00000D000000}" name="DESVIO NOMINAL %" dataDxfId="3" dataCellStyle="Porcentagem">
       <calculatedColumnFormula>IFERROR(Tabela5[[#This Row],[DESVIO NOMINAL R$]]/Tabela5[[#This Row],[VALOR ORÇADO]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0300-00000E000000}" name="DESVIO CORRIGIDO R$" dataDxfId="8" dataCellStyle="Moeda">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0300-00000E000000}" name="DESVIO CORRIGIDO R$" dataDxfId="2" dataCellStyle="Moeda">
       <calculatedColumnFormula>Tabela5[[#This Row],[VALOR ATUALIZADO]]-Tabela5[[#This Row],[CUSTO AO TÉRMINO]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0300-00000F000000}" name="DESVIO CORRIGIDO %" dataDxfId="7" dataCellStyle="Porcentagem">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0300-00000F000000}" name="DESVIO CORRIGIDO %" dataDxfId="1" dataCellStyle="Porcentagem">
       <calculatedColumnFormula>IFERROR(Tabela5[[#This Row],[DESVIO CORRIGIDO R$]]/Tabela5[[#This Row],[VALOR ATUALIZADO]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1064,17 +1067,17 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabela6" displayName="Tabela6" ref="A3:I6" totalsRowShown="0" headerRowDxfId="6" tableBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabela6" displayName="Tabela6" ref="A3:I6" totalsRowShown="0" headerRowDxfId="35" tableBorderDxfId="34">
   <autoFilter ref="A3:I6" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="ÁREA / LOCAL"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="ITEM"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="1º PRAZO" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="PRAZO ATUAL" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="DELTA" dataDxfId="2">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="1º PRAZO" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="PRAZO ATUAL" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="DELTA" dataDxfId="31">
       <calculatedColumnFormula>IF(OR(C4="",D4=""),"",D4-C4)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="STATUS" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="STATUS" dataDxfId="30"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="RESPONSÁVEL"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="OBSERVAÇÃO"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="OCULTAR"/>
@@ -1442,7 +1445,9 @@
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
+      <c r="A8" s="8" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
@@ -1468,13 +1473,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="24"/>
     </row>
     <row r="2" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="26" t="s">
         <v>19</v>
       </c>
       <c r="B2" s="24"/>
@@ -1504,7 +1509,7 @@
       <c r="B6" s="2"/>
     </row>
     <row r="7" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="26" t="s">
         <v>24</v>
       </c>
       <c r="B7" s="24"/>
@@ -1534,7 +1539,7 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="26" t="s">
         <v>28</v>
       </c>
       <c r="B11" s="24"/>
@@ -1589,7 +1594,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="23" t="s">
         <v>32</v>
       </c>
       <c r="B1" s="24"/>
@@ -1662,7 +1667,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="23" t="s">
         <v>40</v>
       </c>
       <c r="B1" s="24"/>
@@ -1775,17 +1780,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
@@ -1926,7 +1931,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="23" t="s">
         <v>50</v>
       </c>
       <c r="B1" s="24"/>
@@ -1945,23 +1950,23 @@
       <c r="O1" s="24"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
-      <c r="O2" s="29"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29"/>
+      <c r="M2" s="29"/>
+      <c r="N2" s="29"/>
+      <c r="O2" s="30"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
@@ -2196,7 +2201,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="23" t="s">
         <v>73</v>
       </c>
       <c r="B1" s="24"/>
@@ -2204,120 +2209,120 @@
       <c r="D1" s="24"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="32"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="33"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="33"/>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="29"/>
+      <c r="A3" s="34"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="30"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="34"/>
+      <c r="A4" s="35"/>
       <c r="B4" s="24"/>
       <c r="C4" s="24"/>
-      <c r="D4" s="35"/>
+      <c r="D4" s="36"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="34"/>
+      <c r="A5" s="35"/>
       <c r="B5" s="24"/>
       <c r="C5" s="24"/>
-      <c r="D5" s="35"/>
+      <c r="D5" s="36"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="34"/>
+      <c r="A6" s="35"/>
       <c r="B6" s="24"/>
       <c r="C6" s="24"/>
-      <c r="D6" s="35"/>
+      <c r="D6" s="36"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="34"/>
+      <c r="A7" s="35"/>
       <c r="B7" s="24"/>
       <c r="C7" s="24"/>
-      <c r="D7" s="35"/>
+      <c r="D7" s="36"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="34"/>
+      <c r="A8" s="35"/>
       <c r="B8" s="24"/>
       <c r="C8" s="24"/>
-      <c r="D8" s="35"/>
+      <c r="D8" s="36"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="34"/>
+      <c r="A9" s="35"/>
       <c r="B9" s="24"/>
       <c r="C9" s="24"/>
-      <c r="D9" s="35"/>
+      <c r="D9" s="36"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="34"/>
+      <c r="A10" s="35"/>
       <c r="B10" s="24"/>
       <c r="C10" s="24"/>
-      <c r="D10" s="35"/>
+      <c r="D10" s="36"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="34"/>
+      <c r="A11" s="35"/>
       <c r="B11" s="24"/>
       <c r="C11" s="24"/>
-      <c r="D11" s="35"/>
+      <c r="D11" s="36"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="34"/>
+      <c r="A12" s="35"/>
       <c r="B12" s="24"/>
       <c r="C12" s="24"/>
-      <c r="D12" s="35"/>
+      <c r="D12" s="36"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="34"/>
+      <c r="A13" s="35"/>
       <c r="B13" s="24"/>
       <c r="C13" s="24"/>
-      <c r="D13" s="35"/>
+      <c r="D13" s="36"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="34"/>
+      <c r="A14" s="35"/>
       <c r="B14" s="24"/>
       <c r="C14" s="24"/>
-      <c r="D14" s="35"/>
+      <c r="D14" s="36"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="34"/>
+      <c r="A15" s="35"/>
       <c r="B15" s="24"/>
       <c r="C15" s="24"/>
-      <c r="D15" s="35"/>
+      <c r="D15" s="36"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="34"/>
+      <c r="A16" s="35"/>
       <c r="B16" s="24"/>
       <c r="C16" s="24"/>
-      <c r="D16" s="35"/>
+      <c r="D16" s="36"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="34"/>
+      <c r="A17" s="35"/>
       <c r="B17" s="24"/>
       <c r="C17" s="24"/>
-      <c r="D17" s="35"/>
+      <c r="D17" s="36"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="34"/>
+      <c r="A18" s="35"/>
       <c r="B18" s="24"/>
       <c r="C18" s="24"/>
-      <c r="D18" s="35"/>
+      <c r="D18" s="36"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="34"/>
+      <c r="A19" s="35"/>
       <c r="B19" s="24"/>
       <c r="C19" s="24"/>
-      <c r="D19" s="35"/>
+      <c r="D19" s="36"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="36"/>
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="38"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="38"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2346,7 +2351,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="24"/>
@@ -2359,7 +2364,7 @@
       <c r="I1" s="24"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="24"/>

</xml_diff>